<commit_message>
Creadas migraciones para UnidadesCurriculares y ComisionUC, avanzado sistema de calificaciones y tareas/materiales
</commit_message>
<xml_diff>
--- a/BACKEND/EjemplosExcels/file-ITI.xlsx
+++ b/BACKEND/EjemplosExcels/file-ITI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\SVS-System\BACKEND\EjemplosExcels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\Nueva carpeta (2)\SVS-System\BACKEND\EjemplosExcels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC229D10-0D2E-4180-9EBE-B2021B1AE112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8EB488-8CBD-408C-9036-D4B30574B815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -172,10 +172,10 @@
     <t>DNI - 99765489</t>
   </si>
   <si>
-    <t>DNI - 49062828</t>
+    <t>2da</t>
   </si>
   <si>
-    <t>2da</t>
+    <t>DNI - 89062828</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -714,7 +714,7 @@
       </c>
       <c r="J3" s="10"/>
       <c r="K3" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -747,7 +747,7 @@
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -782,7 +782,7 @@
         <v>33</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -817,7 +817,7 @@
         <v>33</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -825,7 +825,7 @@
         <v>38</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>18</v>
@@ -850,7 +850,7 @@
       </c>
       <c r="J7" s="10"/>
       <c r="K7" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>